<commit_message>
Import a barcode column from sales/product files
Files may carry a barcode column (barcode, EAN, UPC, GTIN, code barre, ...).
Excel-mangled cells (3017620422003.0, 3.01762E+12, a UPC-A missing its leading
zero) are repaired when the GS1 check digit confirms it; an invalid cell is
ignored and never blocks the sales row.

Promotion records the barcode on products that have none (fill-only, never
overwrites a curated one, never reuses a barcode across products) and treats a
row whose barcode matches an existing product as that product rather than
creating a duplicate under a different POS name. Duplicate-row detection is
unchanged. The distributed import template gains an optional barcode column.
</commit_message>
<xml_diff>
--- a/backend/templates/apex_sales_import_v1.xlsx
+++ b/backend/templates/apex_sales_import_v1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,10 +469,15 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>barcode</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>competitor_name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>amount_raw</t>
         </is>
@@ -531,10 +536,15 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>6221031020018</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>Rival Store</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>66.15</t>
         </is>

</xml_diff>